<commit_message>
Actualiza horarios 25-oct: etiquetas Semana 45-48
</commit_message>
<xml_diff>
--- a/horarios.xlsx
+++ b/horarios.xlsx
@@ -58,7 +58,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -68,17 +68,14 @@
     <xf numFmtId="20" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="16" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="16" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -453,9 +450,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="8" t="inlineStr">
-        <is>
-          <t>Semana 2 · 2 al 8 de noviembre (S45)</t>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Semana 45</t>
         </is>
       </c>
     </row>
@@ -465,25 +462,25 @@
           <t>Promotor</t>
         </is>
       </c>
-      <c r="B2" s="9" t="n">
+      <c r="B2" s="5" t="n">
         <v>46328</v>
       </c>
-      <c r="D2" s="9" t="n">
+      <c r="D2" s="5" t="n">
         <v>46329</v>
       </c>
-      <c r="F2" s="9" t="n">
+      <c r="F2" s="5" t="n">
         <v>46330</v>
       </c>
-      <c r="H2" s="9" t="n">
+      <c r="H2" s="5" t="n">
         <v>46331</v>
       </c>
-      <c r="J2" s="9" t="n">
+      <c r="J2" s="5" t="n">
         <v>46332</v>
       </c>
-      <c r="L2" s="9" t="n">
+      <c r="L2" s="5" t="n">
         <v>46333</v>
       </c>
-      <c r="N2" s="9" t="n">
+      <c r="N2" s="5" t="n">
         <v>46334</v>
       </c>
     </row>
@@ -1358,9 +1355,9 @@
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>Semana 3 · 9 al 15 de noviembre (S46)</t>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Semana 46</t>
         </is>
       </c>
     </row>
@@ -1370,25 +1367,25 @@
           <t>Promotor</t>
         </is>
       </c>
-      <c r="B20" s="9" t="n">
+      <c r="B20" s="5" t="n">
         <v>46335</v>
       </c>
-      <c r="D20" s="9" t="n">
+      <c r="D20" s="5" t="n">
         <v>46336</v>
       </c>
-      <c r="F20" s="9" t="n">
+      <c r="F20" s="5" t="n">
         <v>46337</v>
       </c>
-      <c r="H20" s="9" t="n">
+      <c r="H20" s="5" t="n">
         <v>46338</v>
       </c>
-      <c r="J20" s="9" t="n">
+      <c r="J20" s="5" t="n">
         <v>46339</v>
       </c>
-      <c r="L20" s="9" t="n">
+      <c r="L20" s="5" t="n">
         <v>46340</v>
       </c>
-      <c r="N20" s="9" t="n">
+      <c r="N20" s="5" t="n">
         <v>46341</v>
       </c>
     </row>
@@ -2263,9 +2260,9 @@
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="8" t="inlineStr">
-        <is>
-          <t>Semana 4 · 16 al 22 de noviembre (S47)</t>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Semana 47</t>
         </is>
       </c>
     </row>
@@ -2275,25 +2272,25 @@
           <t>Promotor</t>
         </is>
       </c>
-      <c r="B38" s="9" t="n">
+      <c r="B38" s="5" t="n">
         <v>46342</v>
       </c>
-      <c r="D38" s="9" t="n">
+      <c r="D38" s="5" t="n">
         <v>46343</v>
       </c>
-      <c r="F38" s="9" t="n">
+      <c r="F38" s="5" t="n">
         <v>46344</v>
       </c>
-      <c r="H38" s="9" t="n">
+      <c r="H38" s="5" t="n">
         <v>46345</v>
       </c>
-      <c r="J38" s="9" t="n">
+      <c r="J38" s="5" t="n">
         <v>46346</v>
       </c>
-      <c r="L38" s="9" t="n">
+      <c r="L38" s="5" t="n">
         <v>46347</v>
       </c>
-      <c r="N38" s="9" t="n">
+      <c r="N38" s="5" t="n">
         <v>46348</v>
       </c>
     </row>
@@ -3168,9 +3165,9 @@
       </c>
     </row>
     <row r="55">
-      <c r="B55" s="8" t="inlineStr">
-        <is>
-          <t>Semana 5 · 23 al 29 de noviembre (S48)</t>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>Semana 48</t>
         </is>
       </c>
     </row>
@@ -3180,25 +3177,25 @@
           <t>Promotor</t>
         </is>
       </c>
-      <c r="B56" s="9" t="n">
+      <c r="B56" s="5" t="n">
         <v>46349</v>
       </c>
-      <c r="D56" s="9" t="n">
+      <c r="D56" s="5" t="n">
         <v>46350</v>
       </c>
-      <c r="F56" s="9" t="n">
+      <c r="F56" s="5" t="n">
         <v>46351</v>
       </c>
-      <c r="H56" s="9" t="n">
+      <c r="H56" s="5" t="n">
         <v>46352</v>
       </c>
-      <c r="J56" s="9" t="n">
+      <c r="J56" s="5" t="n">
         <v>46353</v>
       </c>
-      <c r="L56" s="9" t="n">
+      <c r="L56" s="5" t="n">
         <v>46354</v>
       </c>
-      <c r="N56" s="9" t="n">
+      <c r="N56" s="5" t="n">
         <v>46355</v>
       </c>
     </row>
@@ -4077,8 +4074,8 @@
     <mergeCell ref="L2:M2"/>
     <mergeCell ref="D20:E20"/>
     <mergeCell ref="H20:I20"/>
+    <mergeCell ref="N20:O20"/>
     <mergeCell ref="H38:I38"/>
-    <mergeCell ref="N20:O20"/>
     <mergeCell ref="J38:K38"/>
     <mergeCell ref="B56:C56"/>
     <mergeCell ref="H56:I56"/>
@@ -4092,9 +4089,9 @@
     <mergeCell ref="B38:C38"/>
     <mergeCell ref="J20:K20"/>
     <mergeCell ref="H2:I2"/>
+    <mergeCell ref="F38:G38"/>
+    <mergeCell ref="L38:M38"/>
     <mergeCell ref="L20:M20"/>
-    <mergeCell ref="L38:M38"/>
-    <mergeCell ref="F38:G38"/>
     <mergeCell ref="N38:O38"/>
     <mergeCell ref="B19:O19"/>
     <mergeCell ref="B37:O37"/>

</xml_diff>